<commit_message>
Updating BOM of first prototype
</commit_message>
<xml_diff>
--- a/Prototyping/FirstPrototypeBOM.xlsx
+++ b/Prototyping/FirstPrototypeBOM.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="92">
   <si>
     <t>Component/Equipment Name</t>
   </si>
@@ -215,9 +215,6 @@
   </si>
   <si>
     <t>https://www.lem.com/en/product-list/lf-310s</t>
-  </si>
-  <si>
-    <t>https://www.accuenergy.com/products/hv2-dc-voltage-sensor/?utm_source=chatgpt.com</t>
   </si>
   <si>
     <t>DC-Link voltage monitoring (e.g., DVL 1500-UI)</t>
@@ -294,12 +291,30 @@
   <si>
     <t>SiC MOSFETs</t>
   </si>
+  <si>
+    <t>https://www.accuenergy.com/products/hv2-dc-voltage-sensor/</t>
+  </si>
+  <si>
+    <t>https://www.infineon.com/cms/en/product/power/gate-driver-ics/1ed3890mc12m/#!designsupport</t>
+  </si>
+  <si>
+    <t>Imperix VHDCI Breakout PCB</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/Electronics-Salon-68-Pin-SCSI-5-Terminal-Breakout/dp/B07C9X68G6</t>
+  </si>
+  <si>
+    <t>https://se.farnell.com/ni/785633-01/vhdci-connector-68-pin-r-a-tht/dp/3622789?gross_price=true&amp;CMP=KNC-GSE-GEN-Shopping-Pmax-High-ROAS&amp;mckv=_dc|pcrid||&amp;gad_source=1&amp;gclid=CjwKCAiAiaC-BhBEEiwAjY99qOujcMV8-8jrrJwTcc46v-AvITfLAboAL8qO4t8aKMm0DDaEuoLnFBoCJbMQAvD_BwE</t>
+  </si>
+  <si>
+    <t>VHDCI HD68</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -361,6 +376,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -500,12 +523,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -555,351 +579,43 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
     <cellStyle name="Good" xfId="1" builtinId="26"/>
+    <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
+  <dxfs count="17">
     <dxf>
       <fill>
-        <patternFill>
+        <patternFill patternType="solid">
           <bgColor theme="9" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <fill>
@@ -935,6 +651,366 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -950,17 +1026,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:H22" totalsRowShown="0" headerRowDxfId="0" dataDxfId="14" headerRowBorderDxfId="10" tableBorderDxfId="11" totalsRowBorderDxfId="9">
-  <autoFilter ref="A1:H22"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:H24" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13" headerRowBorderDxfId="11" tableBorderDxfId="12" totalsRowBorderDxfId="10">
+  <autoFilter ref="A1:H24"/>
   <tableColumns count="8">
-    <tableColumn id="1" name="Component/Equipment Name" dataDxfId="8"/>
-    <tableColumn id="2" name="Description" dataDxfId="7"/>
-    <tableColumn id="3" name="Quantity Needed" dataDxfId="6"/>
-    <tableColumn id="4" name="Available Quantity" dataDxfId="5"/>
-    <tableColumn id="5" name="Status" dataDxfId="4"/>
-    <tableColumn id="6" name="Supplier" dataDxfId="3"/>
-    <tableColumn id="7" name="Notes" dataDxfId="2"/>
-    <tableColumn id="9" name="Link" dataDxfId="1"/>
+    <tableColumn id="1" name="Component/Equipment Name" dataDxfId="9"/>
+    <tableColumn id="2" name="Description" dataDxfId="8"/>
+    <tableColumn id="3" name="Quantity Needed" dataDxfId="7"/>
+    <tableColumn id="4" name="Available Quantity" dataDxfId="6"/>
+    <tableColumn id="5" name="Status" dataDxfId="5"/>
+    <tableColumn id="6" name="Supplier" dataDxfId="4"/>
+    <tableColumn id="7" name="Notes" dataDxfId="3"/>
+    <tableColumn id="9" name="Link" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1229,7 +1305,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="59.5703125" style="6" customWidth="1"/>
@@ -1266,13 +1342,13 @@
         <v>6</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I1" s="14"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>60</v>
@@ -1311,7 +1387,9 @@
       <c r="G3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="17"/>
+      <c r="H3" s="17" t="s">
+        <v>87</v>
+      </c>
       <c r="I3" s="15"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -1336,7 +1414,7 @@
       <c r="G4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="17" t="s">
+      <c r="H4" s="19" t="s">
         <v>64</v>
       </c>
       <c r="I4" s="15"/>
@@ -1346,7 +1424,7 @@
         <v>14</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C5" s="4">
         <v>1</v>
@@ -1363,8 +1441,8 @@
       <c r="G5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="17" t="s">
-        <v>65</v>
+      <c r="H5" s="19" t="s">
+        <v>86</v>
       </c>
       <c r="I5" s="15"/>
     </row>
@@ -1373,7 +1451,7 @@
         <v>16</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C6" s="4">
         <v>5</v>
@@ -1382,7 +1460,7 @@
         <v>8</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>18</v>
@@ -1435,13 +1513,13 @@
         <v>7</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G8" s="4" t="s">
         <v>26</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I8" s="15"/>
     </row>
@@ -1450,7 +1528,7 @@
         <v>27</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C9" s="4">
         <v>1</v>
@@ -1462,7 +1540,7 @@
         <v>17</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G9" s="4" t="s">
         <v>28</v>
@@ -1475,7 +1553,7 @@
         <v>29</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C10" s="4">
         <v>6</v>
@@ -1487,13 +1565,13 @@
         <v>7</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>30</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I10" s="15"/>
     </row>
@@ -1502,7 +1580,7 @@
         <v>31</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C11" s="4">
         <v>1</v>
@@ -1549,7 +1627,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>36</v>
@@ -1561,7 +1639,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>22</v>
@@ -1585,9 +1663,7 @@
       <c r="D14" s="4">
         <v>0</v>
       </c>
-      <c r="E14" s="4" t="s">
-        <v>7</v>
-      </c>
+      <c r="E14" s="4"/>
       <c r="F14" s="4"/>
       <c r="G14" s="4" t="s">
         <v>40</v>
@@ -1597,7 +1673,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="4">
@@ -1609,7 +1685,7 @@
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H15" s="17"/>
       <c r="I15" s="15"/>
@@ -1731,21 +1807,53 @@
       <c r="H22" s="18"/>
       <c r="I22" s="15"/>
     </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="21"/>
+      <c r="H23" s="18" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="B24" s="21"/>
+      <c r="C24" s="21"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="21"/>
+      <c r="G24" s="21"/>
+      <c r="H24" s="18" t="s">
+        <v>90</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:H22">
-    <cfRule type="expression" dxfId="13" priority="2">
+  <conditionalFormatting sqref="A1:H24">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>"$A$1:$G$31"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:XFD1048576">
-    <cfRule type="expression" dxfId="12" priority="1">
+    <cfRule type="expression" dxfId="16" priority="1">
       <formula>"$A$1:$G$31"</formula>
     </cfRule>
   </conditionalFormatting>
+  <hyperlinks>
+    <hyperlink ref="H5" r:id="rId1"/>
+    <hyperlink ref="H4" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1760,7 +1868,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -1768,22 +1876,22 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Prototyping BOM and presentations
</commit_message>
<xml_diff>
--- a/Prototyping/FirstPrototypeBOM.xlsx
+++ b/Prototyping/FirstPrototypeBOM.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="98">
   <si>
     <t>Component/Equipment Name</t>
   </si>
@@ -308,6 +308,24 @@
   </si>
   <si>
     <t>VHDCI HD68</t>
+  </si>
+  <si>
+    <t>https://se.rs-online.com/web/p/dc-dc-converters/8289040</t>
+  </si>
+  <si>
+    <t>Isolated DC-DC supply</t>
+  </si>
+  <si>
+    <t>Opamp Isolation</t>
+  </si>
+  <si>
+    <t>https://www.ti.com/product/ISO224</t>
+  </si>
+  <si>
+    <t>https://www.ti.com/lit/an/sbaa321a/sbaa321a.pdf?ts=1743507065660&amp;ref_url=https%253A%252F%252Fwww.google.com%252F</t>
+  </si>
+  <si>
+    <t>https://docs.rs-online.com/4e7c/A700000007009511.pdf</t>
   </si>
 </sst>
 </file>
@@ -529,7 +547,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -588,6 +606,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
@@ -595,28 +616,7 @@
     <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="17">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
+  <dxfs count="16">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -986,6 +986,13 @@
     </dxf>
     <dxf>
       <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
         <patternFill patternType="solid">
           <bgColor theme="9" tint="0.39994506668294322"/>
         </patternFill>
@@ -1005,13 +1012,6 @@
         </bottom>
       </border>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1026,17 +1026,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:H24" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13" headerRowBorderDxfId="11" tableBorderDxfId="12" totalsRowBorderDxfId="10">
-  <autoFilter ref="A1:H24"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:H28" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12" headerRowBorderDxfId="10" tableBorderDxfId="11" totalsRowBorderDxfId="9">
+  <autoFilter ref="A1:H28"/>
   <tableColumns count="8">
-    <tableColumn id="1" name="Component/Equipment Name" dataDxfId="9"/>
-    <tableColumn id="2" name="Description" dataDxfId="8"/>
-    <tableColumn id="3" name="Quantity Needed" dataDxfId="7"/>
-    <tableColumn id="4" name="Available Quantity" dataDxfId="6"/>
-    <tableColumn id="5" name="Status" dataDxfId="5"/>
-    <tableColumn id="6" name="Supplier" dataDxfId="4"/>
-    <tableColumn id="7" name="Notes" dataDxfId="3"/>
-    <tableColumn id="9" name="Link" dataDxfId="2"/>
+    <tableColumn id="1" name="Component/Equipment Name" dataDxfId="8"/>
+    <tableColumn id="2" name="Description" dataDxfId="7"/>
+    <tableColumn id="3" name="Quantity Needed" dataDxfId="6"/>
+    <tableColumn id="4" name="Available Quantity" dataDxfId="5"/>
+    <tableColumn id="5" name="Status" dataDxfId="4"/>
+    <tableColumn id="6" name="Supplier" dataDxfId="3"/>
+    <tableColumn id="7" name="Notes" dataDxfId="2"/>
+    <tableColumn id="9" name="Link" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1305,7 +1305,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="59.5703125" style="6" customWidth="1"/>
@@ -1371,7 +1371,7 @@
       <c r="H2" s="17"/>
       <c r="I2" s="15"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>61</v>
       </c>
@@ -1387,7 +1387,7 @@
       <c r="G3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="17" t="s">
+      <c r="H3" s="19" t="s">
         <v>87</v>
       </c>
       <c r="I3" s="15"/>
@@ -1496,7 +1496,7 @@
       <c r="H7" s="17"/>
       <c r="I7" s="15"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>24</v>
       </c>
@@ -1518,7 +1518,7 @@
       <c r="G8" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="H8" s="17" t="s">
+      <c r="H8" s="19" t="s">
         <v>69</v>
       </c>
       <c r="I8" s="15"/>
@@ -1548,7 +1548,7 @@
       <c r="H9" s="17"/>
       <c r="I9" s="15"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>29</v>
       </c>
@@ -1570,7 +1570,7 @@
       <c r="G10" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H10" s="17" t="s">
+      <c r="H10" s="19" t="s">
         <v>73</v>
       </c>
       <c r="I10" s="15"/>
@@ -1807,7 +1807,7 @@
       <c r="H22" s="18"/>
       <c r="I22" s="15"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="20" t="s">
         <v>88</v>
       </c>
@@ -1817,11 +1817,11 @@
       <c r="E23" s="21"/>
       <c r="F23" s="21"/>
       <c r="G23" s="21"/>
-      <c r="H23" s="18" t="s">
+      <c r="H23" s="22" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="78.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A24" s="20" t="s">
         <v>91</v>
       </c>
@@ -1831,29 +1831,89 @@
       <c r="E24" s="21"/>
       <c r="F24" s="21"/>
       <c r="G24" s="21"/>
-      <c r="H24" s="18" t="s">
+      <c r="H24" s="22" t="s">
         <v>90</v>
       </c>
     </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="20"/>
+      <c r="B25" s="21" t="s">
+        <v>93</v>
+      </c>
+      <c r="C25" s="21"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="21"/>
+      <c r="G25" s="21"/>
+      <c r="H25" s="22" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" s="20"/>
+      <c r="B26" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="C26" s="21"/>
+      <c r="D26" s="21"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="21"/>
+      <c r="G26" s="21"/>
+      <c r="H26" s="18" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A27" s="20"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="21"/>
+      <c r="H27" s="18" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="20"/>
+      <c r="B28" s="21" t="s">
+        <v>94</v>
+      </c>
+      <c r="C28" s="21"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="21"/>
+      <c r="H28" s="18" t="s">
+        <v>97</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A1:H24">
-    <cfRule type="expression" dxfId="1" priority="2">
+  <conditionalFormatting sqref="A1:H28">
+    <cfRule type="expression" dxfId="15" priority="2">
       <formula>"$A$1:$G$31"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:XFD1048576">
-    <cfRule type="expression" dxfId="16" priority="1">
+    <cfRule type="expression" dxfId="14" priority="1">
       <formula>"$A$1:$G$31"</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="H5" r:id="rId1"/>
     <hyperlink ref="H4" r:id="rId2"/>
+    <hyperlink ref="H3" r:id="rId3" location="!designsupport"/>
+    <hyperlink ref="H8" display="https://www.mouser.se/ProductDetail/Cornell-Dubilier-CDE/SCD105K162A3Z25-F?qs=59Iuwm0WYIi7PFxKkjFJtg%3D%3D&amp;srsltid=AfmBOoqS60oh50cgeFOKdh_Q2G4ZsFBuBlZ6EXEBZhpKEFhGAWeO2Euy&amp;_gl=1*1i2vxz7*_ga*MTM1NTQ4MTUzNy4xNzM2NDE4NzMw*_ga_15W4STQT4T*MTczNjQxODczMC4xLjEuM"/>
+    <hyperlink ref="H10" r:id="rId4"/>
+    <hyperlink ref="H24" display="https://se.farnell.com/ni/785633-01/vhdci-connector-68-pin-r-a-tht/dp/3622789?gross_price=true&amp;CMP=KNC-GSE-GEN-Shopping-Pmax-High-ROAS&amp;mckv=_dc|pcrid||&amp;gad_source=1&amp;gclid=CjwKCAiAiaC-BhBEEiwAjY99qOujcMV8-8jrrJwTcc46v-AvITfLAboAL8qO4t8aKMm0DDaEuoLnFBoCJbMQ"/>
+    <hyperlink ref="H25" r:id="rId5"/>
+    <hyperlink ref="H23" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>
   <tableParts count="1">
-    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId8"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>